<commit_message>
feat: add applyTotalsStyle function for Excel report formatting and enhance row height handling in JointReportService
</commit_message>
<xml_diff>
--- a/backend/src/template/GST_Payment_Template.xlsx
+++ b/backend/src/template/GST_Payment_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Desktop\own_pr\Kr\kr_ferm\backend\src\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09CAFFEB-6186-45C7-AF49-9F3521589731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{652DACDD-734D-4C37-8D08-AEF2DF1A1893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9B5721B8-0128-4B9E-815E-8C761AC86527}"/>
   </bookViews>
@@ -174,9 +174,6 @@
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -194,6 +191,9 @@
     </xf>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -516,141 +516,143 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="18.44140625" customWidth="1"/>
-    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" customWidth="1"/>
     <col min="6" max="7" width="14.33203125" customWidth="1"/>
     <col min="9" max="9" width="14.5546875" customWidth="1"/>
+    <col min="10" max="10" width="11" customWidth="1"/>
+    <col min="11" max="11" width="11.77734375" customWidth="1"/>
     <col min="13" max="13" width="11.88671875" customWidth="1"/>
     <col min="14" max="14" width="13.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
     </row>
     <row r="3" spans="1:14" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="M3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N3" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="5">
+      <c r="A4" s="4">
         <v>1</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>150036</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="6">
         <f>+SUM(D4:D4)</f>
         <v>150036</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="6">
         <f>+E4*9%</f>
         <v>13503.24</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="6">
         <f>+F4</f>
         <v>13503.24</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="6">
         <v>-0.2</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="6">
         <f>+E4+F4+G4+H4</f>
         <v>177042.27999999997</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="3">
         <v>0</v>
       </c>
-      <c r="K4" s="7">
+      <c r="K4" s="6">
         <f>+SUM(J4:J4)</f>
         <v>0</v>
       </c>
-      <c r="L4" s="7">
+      <c r="L4" s="6">
         <v>0</v>
       </c>
-      <c r="M4" s="7">
+      <c r="M4" s="6">
         <f>+ROUND(E4*1%,0)</f>
         <v>1500</v>
       </c>
-      <c r="N4" s="7">
+      <c r="N4" s="6">
         <f>+I4-(K4+M4+L4)</f>
         <v>175542.27999999997</v>
       </c>

</xml_diff>